<commit_message>
Add a garden natives half-strength note and remaining product docs.
Garden plans now tell people to use Seaweed Secrets and Activ8Mate at half strength on natives and sensitive plants. Also commit the leftover descriptions, decision-logic files, and engine templates.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/plant_doctor_recommendation_engine_template.xlsx
+++ b/plant_doctor_recommendation_engine_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marketing/PD-Product-Guide/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DDBF1E2-845B-064B-A882-7A44DF22DF30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C383807-E16C-C245-946B-F56559121116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="36960" yWindow="500" windowWidth="34200" windowHeight="19960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5021,7 +5021,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="25" spans="1:45" ht="224" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:45" ht="208" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>228</v>
       </c>
@@ -5959,7 +5959,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="32" spans="1:45" ht="224" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:45" ht="208" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>275</v>
       </c>
@@ -6763,7 +6763,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="38" spans="1:44" ht="208" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:44" ht="224" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>317</v>
       </c>
@@ -6899,12 +6899,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="AJ1:AN1"/>
     <mergeCell ref="H1:O1"/>
     <mergeCell ref="P1:T1"/>
     <mergeCell ref="U1:Z1"/>
     <mergeCell ref="AA1:AD1"/>
     <mergeCell ref="AE1:AI1"/>
-    <mergeCell ref="AJ1:AN1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>